<commit_message>
Complete official inflation and sentiment history from supplied August report
</commit_message>
<xml_diff>
--- a/submission/Lab1_Andreus_85/results/tables.xlsx
+++ b/submission/Lab1_Andreus_85/results/tables.xlsx
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="274">
   <si>
     <t xml:space="preserve">Проверка</t>
   </si>
@@ -639,7 +639,13 @@
     <t xml:space="preserve">2026-01</t>
   </si>
   <si>
-    <t xml:space="preserve">Опубликованный ряд: значение не получено</t>
+    <t xml:space="preserve">Опубликованный ряд</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Медианы: 0,1 п. п.; индексы: 1 пункт</t>
   </si>
   <si>
     <t xml:space="preserve">2026-02</t>
@@ -669,9 +675,6 @@
     <t xml:space="preserve">Синтетическая выборка</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-18</t>
-  </si>
-  <si>
     <t xml:space="preserve">Расчеты без промежуточного округления</t>
   </si>
   <si>
@@ -696,7 +699,7 @@
     <t xml:space="preserve">п. п.</t>
   </si>
   <si>
-    <t xml:space="preserve">Официальное значение не получено</t>
+    <t xml:space="preserve">Рассчитано</t>
   </si>
   <si>
     <t xml:space="preserve">Ожидаемая медиана</t>
@@ -3379,125 +3382,237 @@
       <c r="A2" t="s">
         <v>194</v>
       </c>
-      <c r="B2"/>
-      <c r="C2"/>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2"/>
+      <c r="B2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D2" t="n">
+        <v>91</v>
+      </c>
+      <c r="E2" t="n">
+        <v>107</v>
+      </c>
+      <c r="F2" t="n">
+        <v>101</v>
+      </c>
       <c r="G2" t="s">
         <v>195</v>
       </c>
-      <c r="H2"/>
-      <c r="I2"/>
+      <c r="H2" t="s">
+        <v>196</v>
+      </c>
+      <c r="I2" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>196</v>
-      </c>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3"/>
-      <c r="E3"/>
-      <c r="F3"/>
+        <v>198</v>
+      </c>
+      <c r="B3" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>88</v>
+      </c>
+      <c r="E3" t="n">
+        <v>104</v>
+      </c>
+      <c r="F3" t="n">
+        <v>98</v>
+      </c>
       <c r="G3" t="s">
         <v>195</v>
       </c>
-      <c r="H3"/>
-      <c r="I3"/>
+      <c r="H3" t="s">
+        <v>196</v>
+      </c>
+      <c r="I3" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>197</v>
-      </c>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
-      <c r="E4"/>
-      <c r="F4"/>
+        <v>199</v>
+      </c>
+      <c r="B4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="C4" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>88</v>
+      </c>
+      <c r="E4" t="n">
+        <v>105</v>
+      </c>
+      <c r="F4" t="n">
+        <v>98</v>
+      </c>
       <c r="G4" t="s">
         <v>195</v>
       </c>
-      <c r="H4"/>
-      <c r="I4"/>
+      <c r="H4" t="s">
+        <v>196</v>
+      </c>
+      <c r="I4" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>198</v>
-      </c>
-      <c r="B5"/>
-      <c r="C5"/>
-      <c r="D5"/>
-      <c r="E5"/>
-      <c r="F5"/>
+        <v>200</v>
+      </c>
+      <c r="B5" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="C5" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="D5" t="n">
+        <v>85</v>
+      </c>
+      <c r="E5" t="n">
+        <v>101</v>
+      </c>
+      <c r="F5" t="n">
+        <v>94</v>
+      </c>
       <c r="G5" t="s">
         <v>195</v>
       </c>
-      <c r="H5"/>
-      <c r="I5"/>
+      <c r="H5" t="s">
+        <v>196</v>
+      </c>
+      <c r="I5" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>199</v>
-      </c>
-      <c r="B6"/>
-      <c r="C6"/>
-      <c r="D6"/>
-      <c r="E6"/>
-      <c r="F6"/>
+        <v>201</v>
+      </c>
+      <c r="B6" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D6" t="n">
+        <v>89</v>
+      </c>
+      <c r="E6" t="n">
+        <v>102</v>
+      </c>
+      <c r="F6" t="n">
+        <v>96</v>
+      </c>
       <c r="G6" t="s">
         <v>195</v>
       </c>
-      <c r="H6"/>
-      <c r="I6"/>
+      <c r="H6" t="s">
+        <v>196</v>
+      </c>
+      <c r="I6" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>200</v>
-      </c>
-      <c r="B7"/>
-      <c r="C7"/>
-      <c r="D7"/>
-      <c r="E7"/>
-      <c r="F7"/>
+        <v>202</v>
+      </c>
+      <c r="B7" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="D7" t="n">
+        <v>89</v>
+      </c>
+      <c r="E7" t="n">
+        <v>104</v>
+      </c>
+      <c r="F7" t="n">
+        <v>98</v>
+      </c>
       <c r="G7" t="s">
         <v>195</v>
       </c>
-      <c r="H7"/>
-      <c r="I7"/>
+      <c r="H7" t="s">
+        <v>196</v>
+      </c>
+      <c r="I7" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>201</v>
-      </c>
-      <c r="B8"/>
-      <c r="C8"/>
-      <c r="D8"/>
-      <c r="E8"/>
-      <c r="F8"/>
+        <v>203</v>
+      </c>
+      <c r="B8" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E8" t="n">
+        <v>92</v>
+      </c>
+      <c r="F8" t="n">
+        <v>90</v>
+      </c>
       <c r="G8" t="s">
         <v>195</v>
       </c>
-      <c r="H8"/>
-      <c r="I8"/>
+      <c r="H8" t="s">
+        <v>196</v>
+      </c>
+      <c r="I8" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>202</v>
-      </c>
-      <c r="B9"/>
-      <c r="C9"/>
-      <c r="D9"/>
-      <c r="E9"/>
-      <c r="F9"/>
+        <v>204</v>
+      </c>
+      <c r="B9" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D9" t="n">
+        <v>87</v>
+      </c>
+      <c r="E9" t="n">
+        <v>96</v>
+      </c>
+      <c r="F9" t="n">
+        <v>93</v>
+      </c>
       <c r="G9" t="s">
         <v>195</v>
       </c>
-      <c r="H9"/>
-      <c r="I9"/>
+      <c r="H9" t="s">
+        <v>196</v>
+      </c>
+      <c r="I9" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B10" t="n">
         <v>15.1966292134831</v>
@@ -3515,13 +3630,13 @@
         <v>92.89</v>
       </c>
       <c r="G10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="H10" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="I10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -3743,99 +3858,119 @@
         <v>14</v>
       </c>
       <c r="B1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>212</v>
-      </c>
-      <c r="B2"/>
+        <v>213</v>
+      </c>
+      <c r="B2" t="n">
+        <v>14.3</v>
+      </c>
       <c r="C2" t="n">
         <v>15.1966292134831</v>
       </c>
-      <c r="D2"/>
+      <c r="D2" t="n">
+        <v>0.896629213483145</v>
+      </c>
       <c r="E2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>215</v>
-      </c>
-      <c r="B3"/>
+        <v>216</v>
+      </c>
+      <c r="B3" t="n">
+        <v>13.7</v>
+      </c>
       <c r="C3" t="n">
         <v>13.8846153846154</v>
       </c>
-      <c r="D3"/>
+      <c r="D3" t="n">
+        <v>0.184615384615386</v>
+      </c>
       <c r="E3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
         <v>154</v>
       </c>
-      <c r="B4"/>
+      <c r="B4" t="n">
+        <v>87</v>
+      </c>
       <c r="C4" t="n">
         <v>86.3</v>
       </c>
-      <c r="D4"/>
+      <c r="D4" t="n">
+        <v>-0.699999999999989</v>
+      </c>
       <c r="E4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
         <v>155</v>
       </c>
-      <c r="B5"/>
+      <c r="B5" t="n">
+        <v>96</v>
+      </c>
       <c r="C5" t="n">
         <v>97.2833333333333</v>
       </c>
-      <c r="D5"/>
+      <c r="D5" t="n">
+        <v>1.28333333333335</v>
+      </c>
       <c r="E5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
         <v>156</v>
       </c>
-      <c r="B6"/>
+      <c r="B6" t="n">
+        <v>93</v>
+      </c>
       <c r="C6" t="n">
         <v>92.89</v>
       </c>
-      <c r="D6"/>
+      <c r="D6" t="n">
+        <v>-0.109999999999985</v>
+      </c>
       <c r="E6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -3906,7 +4041,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B2" t="n">
         <v>402</v>
@@ -3917,7 +4052,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B3" t="n">
         <v>529</v>
@@ -3928,7 +4063,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B4" t="n">
         <v>573</v>
@@ -3939,7 +4074,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B5" t="n">
         <v>496</v>
@@ -3972,7 +4107,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B2" t="n">
         <v>660</v>
@@ -3983,7 +4118,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B3" t="n">
         <v>78</v>
@@ -3994,7 +4129,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B4" t="n">
         <v>511</v>
@@ -4005,7 +4140,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B5" t="n">
         <v>751</v>
@@ -4038,7 +4173,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B2" t="n">
         <v>88</v>
@@ -4049,7 +4184,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B3" t="n">
         <v>80</v>
@@ -4060,7 +4195,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B4" t="n">
         <v>470</v>
@@ -4071,7 +4206,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B5" t="n">
         <v>1192</v>
@@ -4082,7 +4217,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B6" t="n">
         <v>170</v>
@@ -4115,7 +4250,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B2" t="n">
         <v>506</v>
@@ -4126,7 +4261,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B3" t="n">
         <v>686</v>
@@ -4159,7 +4294,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B2" t="n">
         <v>1423</v>
@@ -4170,7 +4305,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B3" t="n">
         <v>577</v>
@@ -4203,7 +4338,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B2" t="n">
         <v>128</v>
@@ -4214,7 +4349,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B3" t="n">
         <v>361</v>
@@ -4225,7 +4360,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B4" t="n">
         <v>732</v>
@@ -4236,7 +4371,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B5" t="n">
         <v>456</v>
@@ -4247,7 +4382,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B6" t="n">
         <v>323</v>
@@ -4280,7 +4415,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B2" t="n">
         <v>921</v>
@@ -4291,7 +4426,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B3" t="n">
         <v>726</v>
@@ -4302,7 +4437,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B4" t="n">
         <v>169</v>
@@ -4313,7 +4448,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B5" t="n">
         <v>83</v>
@@ -4324,7 +4459,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B6" t="n">
         <v>6</v>
@@ -4368,7 +4503,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B2" t="n">
         <v>396</v>
@@ -4379,7 +4514,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B3" t="n">
         <v>888</v>
@@ -4390,7 +4525,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B4" t="n">
         <v>297</v>
@@ -4401,7 +4536,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B5" t="n">
         <v>189</v>
@@ -4412,7 +4547,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B6" t="n">
         <v>8</v>
@@ -4987,7 +5122,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B2" t="n">
         <v>1113</v>
@@ -4998,7 +5133,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B3" t="n">
         <v>650</v>
@@ -5009,7 +5144,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B4" t="n">
         <v>109</v>
@@ -5020,7 +5155,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B5" t="n">
         <v>19</v>
@@ -5031,7 +5166,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B6" t="n">
         <v>0</v>
@@ -5471,7 +5606,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B2" t="n">
         <v>301</v>
@@ -5482,7 +5617,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B3" t="n">
         <v>1025</v>
@@ -5493,7 +5628,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B4" t="n">
         <v>633</v>
@@ -5537,7 +5672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B2" t="n">
         <v>428</v>
@@ -5548,7 +5683,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B3" t="n">
         <v>751</v>
@@ -5559,7 +5694,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B4" t="n">
         <v>460</v>
@@ -5603,7 +5738,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B2" t="n">
         <v>247</v>
@@ -5614,7 +5749,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B3" t="n">
         <v>363</v>
@@ -5625,7 +5760,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B4" t="n">
         <v>481</v>
@@ -5636,7 +5771,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B5" t="n">
         <v>242</v>
@@ -5647,7 +5782,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B6" t="n">
         <v>432</v>
@@ -5691,7 +5826,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B2" t="n">
         <v>388</v>
@@ -5702,7 +5837,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B3" t="n">
         <v>628</v>
@@ -5713,7 +5848,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B4" t="n">
         <v>455</v>
@@ -5757,7 +5892,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B2" t="n">
         <v>395</v>
@@ -5768,7 +5903,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B3" t="n">
         <v>803</v>
@@ -5779,7 +5914,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B4" t="n">
         <v>611</v>
@@ -6072,7 +6207,7 @@
         <v>52</v>
       </c>
       <c r="C1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2">
@@ -6209,7 +6344,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
@@ -6220,7 +6355,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B15" t="n">
         <v>0</v>
@@ -6231,7 +6366,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B16" t="n">
         <v>128</v>
@@ -6242,7 +6377,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B17" t="n">
         <v>0</v>
@@ -6270,7 +6405,7 @@
         <v>52</v>
       </c>
       <c r="C1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2">
@@ -6407,7 +6542,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
@@ -6418,7 +6553,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B15" t="n">
         <v>0</v>
@@ -6429,7 +6564,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B16" t="n">
         <v>331</v>
@@ -6440,7 +6575,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B17" t="n">
         <v>0</v>

</xml_diff>